<commit_message>
Updated Sprint Review and Teamprotokoll
</commit_message>
<xml_diff>
--- a/Sprint_Review_Protocol_2.xlsx
+++ b/Sprint_Review_Protocol_2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\florian\Desktop\itp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{56567AA2-BCCF-4002-B7BE-D19A3A6C49AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BF56AAD6-A9B9-47C2-B8B2-A269D3628EA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{5C77D34F-34C3-4D2F-849C-09193AE86D67}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="30">
   <si>
     <t>Sprint Review Protocol</t>
   </si>
@@ -111,6 +111,9 @@
   </si>
   <si>
     <t>remarks</t>
+  </si>
+  <si>
+    <t>Sprint/Taschenlampe Funktion</t>
   </si>
   <si>
     <t>…</t>
@@ -371,26 +374,35 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -398,59 +410,50 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -780,168 +783,168 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
-      <c r="G1" s="28"/>
-      <c r="H1" s="28"/>
-      <c r="I1" s="28"/>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
+      <c r="H1" s="11"/>
+      <c r="I1" s="11"/>
     </row>
     <row r="2" spans="1:9">
-      <c r="A2" s="28"/>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
-      <c r="F2" s="28"/>
-      <c r="G2" s="28"/>
-      <c r="H2" s="28"/>
-      <c r="I2" s="28"/>
+      <c r="A2" s="11"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
+      <c r="F2" s="11"/>
+      <c r="G2" s="11"/>
+      <c r="H2" s="11"/>
+      <c r="I2" s="11"/>
     </row>
     <row r="3" spans="1:9" ht="26.25">
-      <c r="A3" s="5"/>
-      <c r="B3" s="5"/>
-      <c r="C3" s="5"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5"/>
-      <c r="H3" s="5"/>
-      <c r="I3" s="5"/>
+      <c r="A3" s="9"/>
+      <c r="B3" s="9"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="9"/>
+      <c r="I3" s="9"/>
     </row>
     <row r="4" spans="1:9">
-      <c r="A4" s="25" t="s">
+      <c r="A4" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="26"/>
-      <c r="C4" s="18">
+      <c r="B4" s="16"/>
+      <c r="C4" s="19">
         <v>2</v>
       </c>
-      <c r="D4" s="18"/>
-      <c r="E4" s="18"/>
-      <c r="F4" s="18"/>
-      <c r="G4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
+      <c r="G4" s="20"/>
     </row>
     <row r="5" spans="1:9">
-      <c r="A5" s="14" t="s">
+      <c r="A5" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="15"/>
-      <c r="C5" s="29">
+      <c r="B5" s="18"/>
+      <c r="C5" s="21">
         <v>46126</v>
       </c>
-      <c r="D5" s="20"/>
-      <c r="E5" s="20"/>
-      <c r="F5" s="20"/>
-      <c r="G5" s="21"/>
+      <c r="D5" s="22"/>
+      <c r="E5" s="22"/>
+      <c r="F5" s="22"/>
+      <c r="G5" s="23"/>
     </row>
     <row r="6" spans="1:9">
-      <c r="A6" s="14" t="s">
+      <c r="A6" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="15"/>
-      <c r="C6" s="20">
+      <c r="B6" s="18"/>
+      <c r="C6" s="22">
         <v>35</v>
       </c>
-      <c r="D6" s="20"/>
-      <c r="E6" s="20"/>
-      <c r="F6" s="20"/>
-      <c r="G6" s="21"/>
+      <c r="D6" s="22"/>
+      <c r="E6" s="22"/>
+      <c r="F6" s="22"/>
+      <c r="G6" s="23"/>
     </row>
     <row r="7" spans="1:9">
-      <c r="A7" s="14" t="s">
+      <c r="A7" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="15"/>
-      <c r="C7" s="30" t="s">
+      <c r="B7" s="18"/>
+      <c r="C7" s="24" t="s">
         <v>5</v>
       </c>
-      <c r="D7" s="22"/>
-      <c r="E7" s="22"/>
-      <c r="F7" s="22"/>
-      <c r="G7" s="23"/>
+      <c r="D7" s="25"/>
+      <c r="E7" s="25"/>
+      <c r="F7" s="25"/>
+      <c r="G7" s="26"/>
     </row>
     <row r="8" spans="1:9">
-      <c r="A8" s="14" t="s">
+      <c r="A8" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="15"/>
-      <c r="C8" s="31" t="s">
+      <c r="B8" s="18"/>
+      <c r="C8" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="D8" s="32"/>
-      <c r="E8" s="32"/>
-      <c r="F8" s="32"/>
-      <c r="G8" s="24"/>
+      <c r="D8" s="13"/>
+      <c r="E8" s="13"/>
+      <c r="F8" s="13"/>
+      <c r="G8" s="14"/>
     </row>
     <row r="9" spans="1:9">
-      <c r="A9" s="14" t="s">
+      <c r="A9" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="15"/>
-      <c r="C9" s="31" t="s">
+      <c r="B9" s="18"/>
+      <c r="C9" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="D9" s="32"/>
-      <c r="E9" s="32"/>
-      <c r="F9" s="32"/>
-      <c r="G9" s="24"/>
+      <c r="D9" s="13"/>
+      <c r="E9" s="13"/>
+      <c r="F9" s="13"/>
+      <c r="G9" s="14"/>
     </row>
     <row r="10" spans="1:9">
-      <c r="A10" s="14" t="s">
+      <c r="A10" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="15"/>
-      <c r="C10" s="31" t="s">
+      <c r="B10" s="18"/>
+      <c r="C10" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="D10" s="32"/>
-      <c r="E10" s="32"/>
-      <c r="F10" s="32"/>
-      <c r="G10" s="24"/>
+      <c r="D10" s="13"/>
+      <c r="E10" s="13"/>
+      <c r="F10" s="13"/>
+      <c r="G10" s="14"/>
     </row>
     <row r="11" spans="1:9">
-      <c r="A11" s="14" t="s">
+      <c r="A11" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="15"/>
-      <c r="C11" s="33" t="s">
+      <c r="B11" s="18"/>
+      <c r="C11" s="27" t="s">
         <v>13</v>
       </c>
-      <c r="D11" s="10"/>
-      <c r="E11" s="10"/>
-      <c r="F11" s="10"/>
-      <c r="G11" s="11"/>
+      <c r="D11" s="28"/>
+      <c r="E11" s="28"/>
+      <c r="F11" s="28"/>
+      <c r="G11" s="29"/>
     </row>
     <row r="12" spans="1:9" ht="16.5" customHeight="1">
-      <c r="A12" s="16" t="s">
+      <c r="A12" s="32" t="s">
         <v>14</v>
       </c>
-      <c r="B12" s="17"/>
-      <c r="C12" s="12" t="s">
+      <c r="B12" s="33"/>
+      <c r="C12" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="D12" s="12"/>
-      <c r="E12" s="12"/>
-      <c r="F12" s="12"/>
-      <c r="G12" s="13"/>
+      <c r="D12" s="30"/>
+      <c r="E12" s="30"/>
+      <c r="F12" s="30"/>
+      <c r="G12" s="31"/>
     </row>
     <row r="14" spans="1:9">
-      <c r="A14" s="27" t="s">
+      <c r="A14" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="B14" s="27"/>
-      <c r="C14" s="27"/>
-      <c r="D14" s="27"/>
-      <c r="E14" s="27"/>
-      <c r="F14" s="27"/>
-      <c r="G14" s="27"/>
-      <c r="H14" s="27"/>
+      <c r="B14" s="10"/>
+      <c r="C14" s="10"/>
+      <c r="D14" s="10"/>
+      <c r="E14" s="10"/>
+      <c r="F14" s="10"/>
+      <c r="G14" s="10"/>
+      <c r="H14" s="10"/>
     </row>
     <row r="15" spans="1:9">
       <c r="A15" s="1" t="s">
@@ -970,190 +973,200 @@
       </c>
     </row>
     <row r="16" spans="1:9">
-      <c r="A16" s="8">
+      <c r="A16" s="7">
         <v>1</v>
       </c>
-      <c r="B16" s="7"/>
-      <c r="C16" s="7"/>
-      <c r="D16" s="7"/>
-      <c r="E16" s="9">
+      <c r="B16" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C16" s="6">
+        <v>2</v>
+      </c>
+      <c r="D16" s="6">
+        <v>4</v>
+      </c>
+      <c r="E16" s="8">
         <f>D16-C16</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F16" s="3"/>
       <c r="G16" s="4"/>
-      <c r="H16" s="7"/>
+      <c r="H16" s="6"/>
     </row>
     <row r="17" spans="1:8">
-      <c r="A17" s="8">
+      <c r="A17" s="7">
         <v>2</v>
       </c>
-      <c r="B17" s="7"/>
-      <c r="C17" s="7"/>
-      <c r="D17" s="7"/>
-      <c r="E17" s="9">
+      <c r="B17" s="6"/>
+      <c r="C17" s="6"/>
+      <c r="D17" s="6"/>
+      <c r="E17" s="8">
         <f t="shared" ref="E17:E25" si="0">D17-C17</f>
         <v>0</v>
       </c>
       <c r="F17" s="3"/>
       <c r="G17" s="4"/>
-      <c r="H17" s="7"/>
+      <c r="H17" s="6"/>
     </row>
     <row r="18" spans="1:8">
-      <c r="A18" s="8">
+      <c r="A18" s="7">
         <v>3</v>
       </c>
-      <c r="B18" s="7"/>
-      <c r="C18" s="7"/>
-      <c r="D18" s="7"/>
-      <c r="E18" s="9">
+      <c r="B18" s="6"/>
+      <c r="C18" s="6"/>
+      <c r="D18" s="6"/>
+      <c r="E18" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F18" s="3"/>
       <c r="G18" s="4"/>
-      <c r="H18" s="7"/>
+      <c r="H18" s="6"/>
     </row>
     <row r="19" spans="1:8">
-      <c r="A19" s="8">
+      <c r="A19" s="7">
         <v>4</v>
       </c>
-      <c r="B19" s="7"/>
-      <c r="C19" s="7"/>
-      <c r="D19" s="7"/>
-      <c r="E19" s="9">
+      <c r="B19" s="6"/>
+      <c r="C19" s="6"/>
+      <c r="D19" s="6"/>
+      <c r="E19" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F19" s="3"/>
       <c r="G19" s="4"/>
-      <c r="H19" s="7"/>
+      <c r="H19" s="6"/>
     </row>
     <row r="20" spans="1:8">
-      <c r="A20" s="8">
+      <c r="A20" s="7">
         <v>5</v>
       </c>
-      <c r="B20" s="7"/>
-      <c r="C20" s="7"/>
-      <c r="D20" s="7"/>
-      <c r="E20" s="9">
+      <c r="B20" s="6"/>
+      <c r="C20" s="6"/>
+      <c r="D20" s="6"/>
+      <c r="E20" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F20" s="3"/>
       <c r="G20" s="4"/>
-      <c r="H20" s="7"/>
+      <c r="H20" s="6"/>
     </row>
     <row r="21" spans="1:8">
-      <c r="A21" s="8">
+      <c r="A21" s="7">
         <v>6</v>
       </c>
-      <c r="B21" s="7"/>
-      <c r="C21" s="7"/>
-      <c r="D21" s="7"/>
-      <c r="E21" s="9">
+      <c r="B21" s="6"/>
+      <c r="C21" s="6"/>
+      <c r="D21" s="6"/>
+      <c r="E21" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F21" s="3"/>
       <c r="G21" s="4"/>
-      <c r="H21" s="7"/>
+      <c r="H21" s="6"/>
     </row>
     <row r="22" spans="1:8">
-      <c r="A22" s="8">
+      <c r="A22" s="7">
         <v>7</v>
       </c>
-      <c r="B22" s="7"/>
-      <c r="C22" s="7"/>
-      <c r="D22" s="7"/>
-      <c r="E22" s="9">
+      <c r="B22" s="6"/>
+      <c r="C22" s="6"/>
+      <c r="D22" s="6"/>
+      <c r="E22" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F22" s="3"/>
       <c r="G22" s="4"/>
-      <c r="H22" s="7"/>
+      <c r="H22" s="6"/>
     </row>
     <row r="23" spans="1:8">
-      <c r="A23" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="B23" s="7"/>
-      <c r="C23" s="7"/>
-      <c r="D23" s="7"/>
-      <c r="E23" s="9">
+      <c r="A23" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B23" s="6"/>
+      <c r="C23" s="6"/>
+      <c r="D23" s="6"/>
+      <c r="E23" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F23" s="3"/>
       <c r="G23" s="4"/>
-      <c r="H23" s="7"/>
+      <c r="H23" s="6"/>
     </row>
     <row r="24" spans="1:8">
-      <c r="A24" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="B24" s="7"/>
-      <c r="C24" s="7"/>
-      <c r="D24" s="7"/>
-      <c r="E24" s="9">
+      <c r="A24" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B24" s="6"/>
+      <c r="C24" s="6"/>
+      <c r="D24" s="6"/>
+      <c r="E24" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F24" s="3"/>
       <c r="G24" s="4"/>
-      <c r="H24" s="7"/>
+      <c r="H24" s="6"/>
     </row>
     <row r="25" spans="1:8">
-      <c r="A25" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="B25" s="7"/>
-      <c r="C25" s="7"/>
-      <c r="D25" s="7"/>
-      <c r="E25" s="9">
+      <c r="A25" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="B25" s="6"/>
+      <c r="C25" s="6"/>
+      <c r="D25" s="6"/>
+      <c r="E25" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F25" s="3"/>
       <c r="G25" s="4"/>
-      <c r="H25" s="7"/>
+      <c r="H25" s="6"/>
     </row>
     <row r="26" spans="1:8">
-      <c r="A26" s="6">
+      <c r="A26" s="5">
         <f>COUNT(A16:A25)</f>
         <v>7</v>
       </c>
-      <c r="B26" s="6"/>
-      <c r="C26" s="6"/>
-      <c r="D26" s="6"/>
-      <c r="E26" s="6">
+      <c r="B26" s="5"/>
+      <c r="C26" s="5"/>
+      <c r="D26" s="5"/>
+      <c r="E26" s="5">
         <f>SUM(E16:E25)</f>
-        <v>0</v>
-      </c>
-      <c r="F26" s="6">
+        <v>2</v>
+      </c>
+      <c r="F26" s="5">
         <f>COUNT(F16:F25)</f>
         <v>0</v>
       </c>
-      <c r="G26" s="6">
+      <c r="G26" s="5">
         <f>COUNT(G16:G25)</f>
         <v>0</v>
       </c>
-      <c r="H26" s="6"/>
+      <c r="H26" s="5"/>
     </row>
     <row r="30" spans="1:8">
-      <c r="A30" s="7"/>
+      <c r="A30" s="6"/>
       <c r="B30" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="31" spans="1:8">
       <c r="B31" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="C12:G12"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="A12:B12"/>
     <mergeCell ref="A14:H14"/>
     <mergeCell ref="A1:I2"/>
     <mergeCell ref="C9:G9"/>
@@ -1170,10 +1183,6 @@
     <mergeCell ref="C7:G7"/>
     <mergeCell ref="C8:G8"/>
     <mergeCell ref="C11:G11"/>
-    <mergeCell ref="C12:G12"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A12:B12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Updated TeamProtokoll and Sprint Review
</commit_message>
<xml_diff>
--- a/Sprint_Review_Protocol_2.xlsx
+++ b/Sprint_Review_Protocol_2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\florian\Desktop\itp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BF56AAD6-A9B9-47C2-B8B2-A269D3628EA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{74FB5ED1-AE38-4D7E-A183-F9A234FD83F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{5C77D34F-34C3-4D2F-849C-09193AE86D67}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="34">
   <si>
     <t>Sprint Review Protocol</t>
   </si>
@@ -111,6 +111,18 @@
   </si>
   <si>
     <t>remarks</t>
+  </si>
+  <si>
+    <t>Sounds implementiert</t>
+  </si>
+  <si>
+    <t>Maplayout, Lichteffekte</t>
+  </si>
+  <si>
+    <t>Objekte/texturen fertiggestellt</t>
+  </si>
+  <si>
+    <t>Enemy Skin/Animation</t>
   </si>
   <si>
     <t>Sprint/Taschenlampe Funktion</t>
@@ -383,6 +395,24 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -404,12 +434,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -442,18 +466,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -783,28 +795,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
-      <c r="H1" s="11"/>
-      <c r="I1" s="11"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
     </row>
     <row r="2" spans="1:9">
-      <c r="A2" s="11"/>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
-      <c r="F2" s="11"/>
-      <c r="G2" s="11"/>
-      <c r="H2" s="11"/>
-      <c r="I2" s="11"/>
+      <c r="A2" s="17"/>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
+      <c r="G2" s="17"/>
+      <c r="H2" s="17"/>
+      <c r="I2" s="17"/>
     </row>
     <row r="3" spans="1:9" ht="26.25">
       <c r="A3" s="9"/>
@@ -818,133 +830,133 @@
       <c r="I3" s="9"/>
     </row>
     <row r="4" spans="1:9">
-      <c r="A4" s="15" t="s">
+      <c r="A4" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="16"/>
-      <c r="C4" s="19">
+      <c r="B4" s="22"/>
+      <c r="C4" s="23">
         <v>2</v>
       </c>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19"/>
-      <c r="G4" s="20"/>
+      <c r="D4" s="23"/>
+      <c r="E4" s="23"/>
+      <c r="F4" s="23"/>
+      <c r="G4" s="24"/>
     </row>
     <row r="5" spans="1:9">
-      <c r="A5" s="17" t="s">
+      <c r="A5" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="18"/>
-      <c r="C5" s="21">
+      <c r="B5" s="13"/>
+      <c r="C5" s="25">
         <v>46126</v>
       </c>
-      <c r="D5" s="22"/>
-      <c r="E5" s="22"/>
-      <c r="F5" s="22"/>
-      <c r="G5" s="23"/>
+      <c r="D5" s="26"/>
+      <c r="E5" s="26"/>
+      <c r="F5" s="26"/>
+      <c r="G5" s="27"/>
     </row>
     <row r="6" spans="1:9">
-      <c r="A6" s="17" t="s">
+      <c r="A6" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="18"/>
-      <c r="C6" s="22">
+      <c r="B6" s="13"/>
+      <c r="C6" s="26">
         <v>35</v>
       </c>
-      <c r="D6" s="22"/>
-      <c r="E6" s="22"/>
-      <c r="F6" s="22"/>
-      <c r="G6" s="23"/>
+      <c r="D6" s="26"/>
+      <c r="E6" s="26"/>
+      <c r="F6" s="26"/>
+      <c r="G6" s="27"/>
     </row>
     <row r="7" spans="1:9">
-      <c r="A7" s="17" t="s">
+      <c r="A7" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="18"/>
-      <c r="C7" s="24" t="s">
+      <c r="B7" s="13"/>
+      <c r="C7" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="D7" s="25"/>
-      <c r="E7" s="25"/>
-      <c r="F7" s="25"/>
-      <c r="G7" s="26"/>
+      <c r="D7" s="29"/>
+      <c r="E7" s="29"/>
+      <c r="F7" s="29"/>
+      <c r="G7" s="30"/>
     </row>
     <row r="8" spans="1:9">
-      <c r="A8" s="17" t="s">
+      <c r="A8" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="18"/>
-      <c r="C8" s="12" t="s">
+      <c r="B8" s="13"/>
+      <c r="C8" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="D8" s="13"/>
-      <c r="E8" s="13"/>
-      <c r="F8" s="13"/>
-      <c r="G8" s="14"/>
+      <c r="D8" s="19"/>
+      <c r="E8" s="19"/>
+      <c r="F8" s="19"/>
+      <c r="G8" s="20"/>
     </row>
     <row r="9" spans="1:9">
-      <c r="A9" s="17" t="s">
+      <c r="A9" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="18"/>
-      <c r="C9" s="12" t="s">
+      <c r="B9" s="13"/>
+      <c r="C9" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="D9" s="13"/>
-      <c r="E9" s="13"/>
-      <c r="F9" s="13"/>
-      <c r="G9" s="14"/>
+      <c r="D9" s="19"/>
+      <c r="E9" s="19"/>
+      <c r="F9" s="19"/>
+      <c r="G9" s="20"/>
     </row>
     <row r="10" spans="1:9">
-      <c r="A10" s="17" t="s">
+      <c r="A10" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="18"/>
-      <c r="C10" s="12" t="s">
+      <c r="B10" s="13"/>
+      <c r="C10" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="D10" s="13"/>
-      <c r="E10" s="13"/>
-      <c r="F10" s="13"/>
-      <c r="G10" s="14"/>
+      <c r="D10" s="19"/>
+      <c r="E10" s="19"/>
+      <c r="F10" s="19"/>
+      <c r="G10" s="20"/>
     </row>
     <row r="11" spans="1:9">
-      <c r="A11" s="17" t="s">
+      <c r="A11" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="18"/>
-      <c r="C11" s="27" t="s">
+      <c r="B11" s="13"/>
+      <c r="C11" s="31" t="s">
         <v>13</v>
       </c>
-      <c r="D11" s="28"/>
-      <c r="E11" s="28"/>
-      <c r="F11" s="28"/>
-      <c r="G11" s="29"/>
+      <c r="D11" s="32"/>
+      <c r="E11" s="32"/>
+      <c r="F11" s="32"/>
+      <c r="G11" s="33"/>
     </row>
     <row r="12" spans="1:9" ht="16.5" customHeight="1">
-      <c r="A12" s="32" t="s">
+      <c r="A12" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="B12" s="33"/>
-      <c r="C12" s="30" t="s">
+      <c r="B12" s="15"/>
+      <c r="C12" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="D12" s="30"/>
-      <c r="E12" s="30"/>
-      <c r="F12" s="30"/>
-      <c r="G12" s="31"/>
+      <c r="D12" s="10"/>
+      <c r="E12" s="10"/>
+      <c r="F12" s="10"/>
+      <c r="G12" s="11"/>
     </row>
     <row r="14" spans="1:9">
-      <c r="A14" s="10" t="s">
+      <c r="A14" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="B14" s="10"/>
-      <c r="C14" s="10"/>
-      <c r="D14" s="10"/>
-      <c r="E14" s="10"/>
-      <c r="F14" s="10"/>
-      <c r="G14" s="10"/>
-      <c r="H14" s="10"/>
+      <c r="B14" s="16"/>
+      <c r="C14" s="16"/>
+      <c r="D14" s="16"/>
+      <c r="E14" s="16"/>
+      <c r="F14" s="16"/>
+      <c r="G14" s="16"/>
+      <c r="H14" s="16"/>
     </row>
     <row r="15" spans="1:9">
       <c r="A15" s="1" t="s">
@@ -980,13 +992,13 @@
         <v>25</v>
       </c>
       <c r="C16" s="6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D16" s="6">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E16" s="8">
-        <f>D16-C16</f>
+        <f>D20-C20</f>
         <v>2</v>
       </c>
       <c r="F16" s="3"/>
@@ -997,12 +1009,18 @@
       <c r="A17" s="7">
         <v>2</v>
       </c>
-      <c r="B17" s="6"/>
-      <c r="C17" s="6"/>
-      <c r="D17" s="6"/>
+      <c r="B17" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C17" s="6">
+        <v>5</v>
+      </c>
+      <c r="D17" s="6">
+        <v>7</v>
+      </c>
       <c r="E17" s="8">
         <f t="shared" ref="E17:E25" si="0">D17-C17</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F17" s="3"/>
       <c r="G17" s="4"/>
@@ -1012,12 +1030,18 @@
       <c r="A18" s="7">
         <v>3</v>
       </c>
-      <c r="B18" s="6"/>
-      <c r="C18" s="6"/>
-      <c r="D18" s="6"/>
+      <c r="B18" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C18" s="6">
+        <v>4</v>
+      </c>
+      <c r="D18" s="6">
+        <v>9</v>
+      </c>
       <c r="E18" s="8">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F18" s="3"/>
       <c r="G18" s="4"/>
@@ -1027,12 +1051,18 @@
       <c r="A19" s="7">
         <v>4</v>
       </c>
-      <c r="B19" s="6"/>
-      <c r="C19" s="6"/>
-      <c r="D19" s="6"/>
+      <c r="B19" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C19" s="6">
+        <v>4</v>
+      </c>
+      <c r="D19" s="6">
+        <v>5</v>
+      </c>
       <c r="E19" s="8">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F19" s="3"/>
       <c r="G19" s="4"/>
@@ -1042,12 +1072,17 @@
       <c r="A20" s="7">
         <v>5</v>
       </c>
-      <c r="B20" s="6"/>
-      <c r="C20" s="6"/>
-      <c r="D20" s="6"/>
+      <c r="B20" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C20" s="6">
+        <v>2</v>
+      </c>
+      <c r="D20" s="6">
+        <v>4</v>
+      </c>
       <c r="E20" s="8">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F20" s="3"/>
       <c r="G20" s="4"/>
@@ -1085,7 +1120,7 @@
     </row>
     <row r="23" spans="1:8">
       <c r="A23" s="7" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="B23" s="6"/>
       <c r="C23" s="6"/>
@@ -1100,7 +1135,7 @@
     </row>
     <row r="24" spans="1:8">
       <c r="A24" s="7" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="B24" s="6"/>
       <c r="C24" s="6"/>
@@ -1115,7 +1150,7 @@
     </row>
     <row r="25" spans="1:8">
       <c r="A25" s="7" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B25" s="6"/>
       <c r="C25" s="6"/>
@@ -1138,7 +1173,7 @@
       <c r="D26" s="5"/>
       <c r="E26" s="5">
         <f>SUM(E16:E25)</f>
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="F26" s="5">
         <f>COUNT(F16:F25)</f>
@@ -1153,21 +1188,16 @@
     <row r="30" spans="1:8">
       <c r="A30" s="6"/>
       <c r="B30" s="2" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
     </row>
     <row r="31" spans="1:8">
       <c r="B31" s="2" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="C12:G12"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="A14:H14"/>
     <mergeCell ref="A1:I2"/>
     <mergeCell ref="C9:G9"/>
     <mergeCell ref="C10:G10"/>
@@ -1182,6 +1212,11 @@
     <mergeCell ref="C6:G6"/>
     <mergeCell ref="C7:G7"/>
     <mergeCell ref="C8:G8"/>
+    <mergeCell ref="C12:G12"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A14:H14"/>
     <mergeCell ref="C11:G11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>

</xml_diff>